<commit_message>
feat: complete Skillbird consolidation milestone
Rename the package/CLI to aimagician_superpower and skillbird, quarantine external sources by default, add category-based install/search and owned skill formatting, consolidate owned workflow/document skills, and record v4 planning plus acceptance evidence.
</commit_message>
<xml_diff>
--- a/skills/owned/window-pptx/templates/template-library/template-library-review.xlsx
+++ b/skills/owned/window-pptx/templates/template-library/template-library-review.xlsx
@@ -92,134 +92,219 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr" s="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TemplateID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>SourcePPTX</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>SlideNo</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>SlideCountInDeck</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PreviewPath</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>VisibleTextSummary</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>ContentSlots</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>StructureTag</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>AIInitialTags</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>HumanReviewedTags</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="1">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>BestFor</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr" s="1">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>AvoidFor</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr" s="1">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>QualityScore</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr" s="1">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ReuseComplexity</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr" s="1">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>EditabilityRisk</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr" s="1">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>ReviewStatus</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr" s="1">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>UseCount</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr" s="1">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>SelectedCount</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr" s="1">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>FinalUsedCount</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr" s="1">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>SelectedRate</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr" s="1">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>FinalUsedRate</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr" s="1">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>CompositeScore</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr" s="1">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Reviewer</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr" s="1">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>LastReviewedDate</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr" s="1">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>PreviewUpdatedAt</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>ShapeCount</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>ImageCount</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>TableCount</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>ChartCount</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>IngestStatus</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>IngestIssue</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>LastAutoIngestedAt</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>VisualLayoutSummary</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>MatchKeywords</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>AIRecommendationReason</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>SuggestedAdaptation</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>RequiredInputs</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>RiskNotes</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>AIQualityReason</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>AutoRecommendStatus</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>ManualLock</t>
         </is>
       </c>
     </row>
@@ -239,25 +324,29 @@
           <t>templates/template-library/reference/封面模板.pptx</t>
         </is>
       </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t/>
+          <t>templates/template-library/previews/0071cf2c__S001.png</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t/>
+          <t>第十九届“挑战杯”全国大学生课外学术科技作品竞赛 健 康 信 息 的 虚 假 革 命 AIGC在虚假信息传播中的作用 AIGC 项目成员：深圳市高端广告设计有限公司 指导老师：深圳市高端广告设计有限公司</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>title, subtitle, visual hero</t>
+          <t>标题, 副标题, 日期/Logo 可选</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -267,7 +356,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>封面模板, 开场页</t>
+          <t>封面模板, 开场页, 标题页</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -282,18 +371,22 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>正文页、数据密集页</t>
-        </is>
-      </c>
-      <c r="N2">
-        <v>4</v>
-      </c>
-      <c r="O2">
-        <v>2</v>
+          <t>正文页、数据密集页、多模块说明页</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -301,14 +394,20 @@
           <t>已通过</t>
         </is>
       </c>
-      <c r="R2">
-        <v>0</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2">
-        <v>0</v>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="U2">
         <f>IF(R2=0,0,S2/R2)</f>
@@ -334,6 +433,91 @@
           <t>V1 seed sample</t>
         </is>
       </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>2026-06-01T16:02:15</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>2026-06-01T16:02:15</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>基于类别、可见文本和对象统计自动初标；形状 21 个，图片 3 个，表格 0 个，图表 0 个，复杂度 中。</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>封面, 标题, 开场, 主题, cover, title</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>类别为 封面模板，结构与该类模板库来源匹配；可见文本和对象统计已完成入库。</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>替换主标题、副标题和品牌信息，并统一当前 deck 主色。</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>主标题；副标题、日期、Logo 可选</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>初始评分来自类别匹配、形状复杂度、图片/表格/图表数量和入库状态；当前状态：AutoRecommendable。</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>AutoRecommendable</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -351,25 +535,29 @@
           <t>templates/template-library/reference/一段内容.pptx</t>
         </is>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t/>
+          <t>templates/template-library/previews/67941e35__S001.png</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t/>
+          <t>请输入大标题 输入标题内容 输入正文内容输入正文内容输入正文内容输入正文内容输入正文内容 输入正文内容输入正文内容输入正文内容输入正文内容输入正文内容 输入正文内容输入正文内容输入正文内容输入正文内容输入正文内容</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>title, one body paragraph</t>
+          <t>标题, 单段正文</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -379,7 +567,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>一段内容, 单段正文</t>
+          <t>一段内容, 单段正文, 介绍页</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -389,19 +577,23 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>简短介绍页、观点页、摘要页</t>
+          <t>简短介绍页、观点页、摘要页、一段正文说明</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>长文、多模块页</t>
-        </is>
-      </c>
-      <c r="N3">
-        <v>4</v>
-      </c>
-      <c r="O3">
-        <v>2</v>
+          <t>长文、多模块并列、复杂数据页</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -413,14 +605,20 @@
           <t>已通过</t>
         </is>
       </c>
-      <c r="R3">
-        <v>0</v>
-      </c>
-      <c r="S3">
-        <v>0</v>
-      </c>
-      <c r="T3">
-        <v>0</v>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="U3">
         <f>IF(R3=0,0,S3/R3)</f>
@@ -446,6 +644,91 @@
           <t>V1 seed sample</t>
         </is>
       </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>2026-06-01T16:02:15</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>2026-06-01T16:02:15</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>基于类别、可见文本和对象统计自动初标；形状 18 个，图片 0 个，表格 0 个，图表 0 个，复杂度 中。</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>一段内容, 正文, 介绍, 摘要, paragraph, body</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>类别为 一段内容，结构与该类模板库来源匹配；可见文本和对象统计已完成入库。</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>替换标题和正文，正文过长时先压缩为一段核心观点。</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>标题；一段 60-140 字左右正文</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>初始评分来自类别匹配、形状复杂度、图片/表格/图表数量和入库状态；当前状态：AutoRecommendable。</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>AutoRecommendable</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -463,25 +746,29 @@
           <t>templates/template-library/reference/人物介绍.pptx</t>
         </is>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t/>
+          <t>templates/template-library/previews/3ff6ed09__S001.png</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t/>
+          <t>李明辉 人工智能领域的资深研究员 创新科技公司的首席技术官（CTO） “每一个伟大的梦想，都始于一个勇敢的开始。在科技的世界里，创新是我们前行的灯塔，照亮未知的领域，引领我们走向更智能、更美好的未来。” LOGO 输入大标题</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>portrait, name, title, bio</t>
+          <t>姓名, 职位/身份, 简介, 照片可选</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -491,7 +778,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>人物介绍, 个人介绍</t>
+          <t>人物介绍, 个人介绍, 团队介绍</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -501,23 +788,27 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>个人介绍、讲师介绍、团队成员页</t>
+          <t>个人介绍、团队成员介绍、嘉宾/讲师介绍</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>无人物素材、数据密集页</t>
-        </is>
-      </c>
-      <c r="N4">
-        <v>4</v>
-      </c>
-      <c r="O4">
-        <v>2</v>
+          <t>纯数据页、流程页、无人物主体的内容页</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -525,14 +816,20 @@
           <t>已通过</t>
         </is>
       </c>
-      <c r="R4">
-        <v>0</v>
-      </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
-      <c r="T4">
-        <v>0</v>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="U4">
         <f>IF(R4=0,0,S4/R4)</f>
@@ -558,6 +855,91 @@
           <t>V1 seed sample</t>
         </is>
       </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>2026-06-01T16:02:15</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>2026-06-01T16:02:15</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>基于类别、可见文本和对象统计自动初标；形状 12 个，图片 2 个，表格 0 个，图表 0 个，复杂度 低。</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>人物, 个人介绍, 团队, 简历, profile, bio</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>类别为 人物介绍，结构与该类模板库来源匹配；可见文本和对象统计已完成入库。</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>替换姓名、身份、简介和头像，并保持人物信息层级清晰。</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>姓名；身份/职位；简介；头像可选</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>初始评分来自类别匹配、形状复杂度、图片/表格/图表数量和入库状态；当前状态：AutoRecommendable。</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>AutoRecommendable</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -575,25 +957,29 @@
           <t>templates/template-library/reference/六段内容.pptx</t>
         </is>
       </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t/>
+          <t>templates/template-library/previews/ade7d363__S001.png</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t/>
+          <t>请输入大标题 LOGO</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>six cards / six modules</t>
+          <t>标题, 六个要点/模块</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -603,7 +989,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>六段内容, 六个要点</t>
+          <t>六段内容, 六项并列, 模块页</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -613,19 +999,23 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>六个模块、六个要点、功能列表</t>
+          <t>6 个要点、6 个模块、6 项能力或 6 步说明</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>少于三点的低密度内容</t>
-        </is>
-      </c>
-      <c r="N5">
-        <v>4</v>
-      </c>
-      <c r="O5">
-        <v>2</v>
+          <t>少于 4 项的内容、长段正文、单一重点页</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -637,14 +1027,20 @@
           <t>已通过</t>
         </is>
       </c>
-      <c r="R5">
-        <v>0</v>
-      </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
-      <c r="T5">
-        <v>0</v>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="U5">
         <f>IF(R5=0,0,S5/R5)</f>
@@ -670,9 +1066,94 @@
           <t>V1 seed sample</t>
         </is>
       </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>2026-06-01T16:02:15</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>2026-06-01T16:02:15</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>基于类别、可见文本和对象统计自动初标；形状 9 个，图片 0 个，表格 0 个，图表 0 个，复杂度 低。</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>六段, 六个要点, 六项, 模块, 6 points, six modules</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>类别为 六段内容，结构与该类模板库来源匹配；可见文本和对象统计已完成入库。</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>把内容压缩成 6 个平行短句，并统一每项标题长度。</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>标题；6 个并列要点或模块名称</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>初始评分来自类别匹配、形状复杂度、图片/表格/图表数量和入库状态；当前状态：AutoRecommendable。</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>AutoRecommendable</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z5"/>
+  <autoFilter ref="A1:AQ5"/>
   <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B200">
       <formula1>"封面模板,一段内容,人物介绍,六段内容"</formula1>

</xml_diff>